<commit_message>
fix(ipa): alinear numeracion de cuadrantes 1, 2, 3, 4 con presentacion oficial CIER
</commit_message>
<xml_diff>
--- a/data/processed/evolucion_importancia_relativa_2025_2026.xlsx
+++ b/data/processed/evolucion_importancia_relativa_2025_2026.xlsx
@@ -624,32 +624,32 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -726,32 +726,32 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -828,32 +828,32 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -930,32 +930,32 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1032,32 +1032,32 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -1134,32 +1134,32 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1236,32 +1236,32 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -1338,32 +1338,32 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1440,32 +1440,32 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1542,12 +1542,12 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1557,17 +1557,17 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1644,32 +1644,32 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -1746,27 +1746,27 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
@@ -1848,27 +1848,27 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -1965,12 +1965,12 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2052,32 +2052,32 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -2154,32 +2154,32 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -2256,27 +2256,27 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2358,27 +2358,27 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
@@ -2460,12 +2460,12 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -2562,32 +2562,32 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -2664,12 +2664,12 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
@@ -2679,12 +2679,12 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -2781,12 +2781,12 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -2868,32 +2868,32 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -2970,32 +2970,32 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -3072,12 +3072,12 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -3087,12 +3087,12 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -3174,32 +3174,32 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -3276,27 +3276,27 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
@@ -3378,32 +3378,32 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -3480,32 +3480,32 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -3582,32 +3582,32 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -5033,32 +5033,32 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -5135,32 +5135,32 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -5237,32 +5237,32 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -5339,32 +5339,32 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -5441,32 +5441,32 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -5543,32 +5543,32 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -5645,32 +5645,32 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
     </row>
@@ -5747,32 +5747,32 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -5849,32 +5849,32 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -5951,12 +5951,12 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -5966,17 +5966,17 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -6053,32 +6053,32 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
     </row>
@@ -6155,27 +6155,27 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -6257,27 +6257,27 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
@@ -6359,12 +6359,12 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
@@ -6374,12 +6374,12 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -6461,32 +6461,32 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Cuadrante IV: Alto Impacto de Mejoras (1º Orden de Intervención)</t>
+          <t>Cuadrante I: Cuadrante Foco / Alto Impacto (1º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Cuadrante IV</t>
+          <t>Cuadrante I</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1º Orden de Intervención - Mejoras graduales y escalables destacadas</t>
+          <t>1º Orden de Intervención - Cuadrante Foco (Mejoras graduales y escalables destacadas)</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -6563,32 +6563,32 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -6665,27 +6665,27 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -6767,27 +6767,27 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Cuadrante I: Fortalezas Clave (2º Orden - Prioridad para MANTENER)</t>
+          <t>Cuadrante III: Fortalezas Clave (2º Orden de Intervención - Prioridad para MANTENER)</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>Cuadrante I</t>
+          <t>Cuadrante III</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2º Orden de Intervención - Prioridad para MANTENER</t>
+          <t>2º Orden de Intervención - Prioridad para MANTENER (Pilares rectores)</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -6869,12 +6869,12 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
@@ -6971,32 +6971,32 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7073,12 +7073,12 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -7088,12 +7088,12 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
@@ -7175,12 +7175,12 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
@@ -7190,12 +7190,12 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -7277,32 +7277,32 @@
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7379,32 +7379,32 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7481,12 +7481,12 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -7496,12 +7496,12 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
@@ -7583,32 +7583,32 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7685,27 +7685,27 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Cuadrante II: Ventajas Secundarias (3º Orden de Intervención)</t>
+          <t>Cuadrante IV: Ventajas Secundarias (3º Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Cuadrante II</t>
+          <t>Cuadrante IV</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
@@ -7787,32 +7787,32 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7889,32 +7889,32 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>
@@ -7991,32 +7991,32 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>Cuadrante III: Baja Prioridad (Último Orden de Intervención)</t>
+          <t>Cuadrante II: Baja Prioridad (Último Orden de Intervención)</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Cuadrante III</t>
+          <t>Cuadrante II</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Último Orden de Intervención - Monitoreo</t>
+          <t>Último Orden de Intervención - Monitoreo sin asignación intensiva</t>
         </is>
       </c>
     </row>

</xml_diff>